<commit_message>
1049192: React Spreadsheet Form Control Sample
</commit_message>
<xml_diff>
--- a/server-side/Files/formControls.xlsx
+++ b/server-side/Files/formControls.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DeiraRajRajkumar\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05A80B63-FB7C-4349-B4F2-14BA6E02CF93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D546380-C6C5-48ED-BF0A-6DE6955AC3DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{26F7903E-E9F7-43B1-BBF4-83CFDB7507BC}"/>
   </bookViews>
@@ -172,7 +172,11 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp6.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="31" fmlaRange="$E$5:$E$13" noThreeD="1" sel="2"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="31" fmlaLink="$G$2:$G$5" fmlaRange="$E$5:$E$13" noThreeD="1" sel="0"/>
+</file>
+
+<file path=xl/ctrlProps/ctrlProp7.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Radio" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -182,15 +186,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>38100</xdr:colOff>
+          <xdr:colOff>44450</xdr:colOff>
           <xdr:row>4</xdr:row>
-          <xdr:rowOff>6350</xdr:rowOff>
+          <xdr:rowOff>25400</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>1797050</xdr:colOff>
+          <xdr:colOff>1104900</xdr:colOff>
           <xdr:row>4</xdr:row>
-          <xdr:rowOff>177800</xdr:rowOff>
+          <xdr:rowOff>171450</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -659,6 +663,92 @@
               </a:ext>
             </a:extLst>
           </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>69850</xdr:colOff>
+          <xdr:row>6</xdr:row>
+          <xdr:rowOff>38100</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>1174750</xdr:colOff>
+          <xdr:row>6</xdr:row>
+          <xdr:rowOff>165100</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1032" name="Option Button 8" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1032"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000008040000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+                <a14:hiddenLine w="9525">
+                  <a:solidFill>
+                    <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+                  </a:solidFill>
+                  <a:miter lim="800000"/>
+                  <a:headEnd/>
+                  <a:tailEnd/>
+                </a14:hiddenLine>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="36576" tIns="32004" rIns="0" bIns="32004" anchor="ctr" upright="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="l" rtl="0">
+                <a:defRPr sz="1000"/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="Segoe UI"/>
+                  <a:cs typeface="Segoe UI"/>
+                </a:rPr>
+                <a:t>Option Button 8</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
         </xdr:sp>
         <xdr:clientData/>
       </xdr:twoCellAnchor>
@@ -986,7 +1076,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B0B0848-7A7E-45E0-B362-58759AA08066}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:Z12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="27.6328125" customWidth="1"/>
@@ -995,7 +1085,7 @@
     <col min="5" max="5" width="14.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="66" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:26" ht="66" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1004,8 +1094,11 @@
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
+      <c r="Z1">
+        <v>7</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1013,7 +1106,7 @@
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
@@ -1029,42 +1122,42 @@
       </c>
       <c r="F3" s="2"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:26" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E5" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.35">
       <c r="E6" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.35">
       <c r="E7" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.35">
       <c r="E8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.35">
       <c r="E9" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.35">
       <c r="E10" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.35">
       <c r="E11" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.35">
       <c r="E12" t="s">
         <v>8</v>
       </c>
@@ -1087,15 +1180,15 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>0</xdr:col>
-                    <xdr:colOff>38100</xdr:colOff>
+                    <xdr:colOff>44450</xdr:colOff>
                     <xdr:row>4</xdr:row>
-                    <xdr:rowOff>6350</xdr:rowOff>
+                    <xdr:rowOff>25400</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>0</xdr:col>
-                    <xdr:colOff>1797050</xdr:colOff>
+                    <xdr:colOff>1104900</xdr:colOff>
                     <xdr:row>4</xdr:row>
-                    <xdr:rowOff>177800</xdr:rowOff>
+                    <xdr:rowOff>171450</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -1212,6 +1305,28 @@
             </control>
           </mc:Choice>
         </mc:AlternateContent>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="1032" r:id="rId10" name="Option Button 8">
+              <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
+                <anchor moveWithCells="1">
+                  <from>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>69850</xdr:colOff>
+                    <xdr:row>6</xdr:row>
+                    <xdr:rowOff>38100</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>1174750</xdr:colOff>
+                    <xdr:row>6</xdr:row>
+                    <xdr:rowOff>165100</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
       </controls>
     </mc:Choice>
   </mc:AlternateContent>

</xml_diff>